<commit_message>
v5.10.0: Market Overview 52-week range, 10-day RSI, Fed Funds and CPI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,12 +450,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
+          <t>Dow Jones</t>
         </is>
       </c>
     </row>
@@ -467,12 +467,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nasdaq 100</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
     </row>
@@ -484,12 +484,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VIX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Volatility</t>
+          <t>Nasdaq 100</t>
         </is>
       </c>
     </row>
@@ -501,12 +501,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dow Jones</t>
+          <t>Russell 2000</t>
         </is>
       </c>
     </row>
@@ -518,36 +518,36 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RSP</t>
+          <t>VIX</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>S&amp;P 500 Equal Weight</t>
+          <t>Volatility</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Broad Market</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Russell 2000</t>
+          <t>Total World</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Broad Market</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -564,7 +564,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Broad Market</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -581,306 +581,306 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Broad Market</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>BND</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Long-Term Bonds</t>
+          <t>US Total Bond</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Broad Market</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IJR</t>
+          <t>BNDX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Small-Cap</t>
+          <t>International Bonds</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Bond Funds</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VBR</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Small-Cap Value</t>
+          <t>20+ Year Treasuries</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Indices</t>
+          <t>Bond Funds</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IJH</t>
+          <t>VGLT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mid-Cap</t>
+          <t>Long-Term Treasuries</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Bond Funds</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VUG</t>
+          <t>VGIT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Intermediate Treasuries</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Bond Funds</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VTV</t>
+          <t>VGSH</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Short-Term Treasuries</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Bond Funds</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VIG</t>
+          <t>VTEB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dividend</t>
+          <t>Tax-Exempt Munis</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SPMO</t>
+          <t>RSP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>S&amp;P 500 Equal Weight</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SPHB</t>
+          <t>IJH</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>High Beta</t>
+          <t>Mid-Cap</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Factors</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SPLV</t>
+          <t>IJR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Low Volatility</t>
+          <t>Small-Cap</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>VBR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Small-Cap Value</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>TOPT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Top 20 Mega-Cap</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>VUG</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Growth</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>VTV</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>VIG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Dividend</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>SPMO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Momentum</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>SPHB</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>High Beta</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Factors</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>SPLV</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Low Volatility</t>
         </is>
       </c>
     </row>
@@ -892,505 +892,505 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Oil (WTI Crude)</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Natural Gas</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Platinum</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HG</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Financials</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2-Year</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>US10Y</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10-Year</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>US30Y</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>30-Year</t>
+          <t>Oil (WTI Crude)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TQQQ</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3x Nasdaq 100</t>
+          <t>Natural Gas</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>3x Semiconductors</t>
+          <t>Gold</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SPXL</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>3x S&amp;P 500</t>
+          <t>Silver</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3x Small-Cap</t>
+          <t>Platinum</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>UDOW</t>
+          <t>HG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3x Dow Jones</t>
+          <t>Copper</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TECL</t>
+          <t>FEDFUNDS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3x Technology</t>
+          <t>Fed Funds Rate</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2x Nasdaq 100</t>
+          <t>2-Year</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SSO</t>
+          <t>US10Y</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2x S&amp;P 500</t>
+          <t>10-Year</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>US30Y</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2x Semiconductors</t>
+          <t>30-Year</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>CPI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>CPI (YoY)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>CORECPI</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Core CPI (YoY)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>TQQQ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>3x Nasdaq 100</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>3x Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>SPXL</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>3x S&amp;P 500</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TRX</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tron</t>
+          <t>3x Small-Cap</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>DOGE</t>
+          <t>UDOW</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dogecoin</t>
+          <t>3x Dow Jones</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ZEC</t>
+          <t>TECL</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Zcash</t>
+          <t>3x Technology</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Cardano</t>
+          <t>2x Nasdaq 100</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>XMR</t>
+          <t>SSO</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Monero</t>
+          <t>2x S&amp;P 500</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LTC</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Litecoin</t>
+          <t>2x Semiconductors</t>
         </is>
       </c>
     </row>
@@ -1402,10 +1402,197 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BNB</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Ripple</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TRX</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Tron</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DOGE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Dogecoin</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ZEC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Zcash</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Cardano</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>XMR</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Monero</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>LTC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Litecoin</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>AVAX</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>

</xml_diff>

<commit_message>
v5.10.1: Market Overview Market Cap category and shorter names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -693,48 +693,48 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tax-Exempt Munis</t>
+          <t>Muni Bonds</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Market Cap</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RSP</t>
+          <t>TOPT</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>S&amp;P 500 Equal Weight</t>
+          <t>Top 20 Mega-Cap</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Market Cap</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IJH</t>
+          <t>RSP</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mid-Cap</t>
+          <t>S&amp;P 500 Equal Weight</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Market Cap</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Market Cap</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -768,17 +768,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Market Cap</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TOPT</t>
+          <t>IJH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Top 20 Mega-Cap</t>
+          <t>Mid-Cap</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CPI (YoY)</t>
+          <t>CPI</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Core CPI (YoY)</t>
+          <t>Core CPI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.10.2: Market Overview Bonds order, Core CPI shown as Core
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -1147,12 +1147,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FEDFUNDS</t>
+          <t>CORECPI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fed Funds Rate</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>CPI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2-Year</t>
+          <t>CPI</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>US10Y</t>
+          <t>FEDFUNDS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10-Year</t>
+          <t>Fed Funds Rate</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>US30Y</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>30-Year</t>
+          <t>2-Year</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1215,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CPI</t>
+          <t>US10Y</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CPI</t>
+          <t>10-Year</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CORECPI</t>
+          <t>US30Y</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Core CPI</t>
+          <t>30-Year</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.10.3: Market Overview adds SMH to Industries
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -909,12 +909,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Semiconductors</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -960,12 +960,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
@@ -994,12 +994,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1011,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
     </row>
@@ -1028,29 +1028,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Industries</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Oil (WTI Crude)</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1062,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Natural Gas</t>
+          <t>Oil (WTI Crude)</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Natural Gas</t>
         </is>
       </c>
     </row>
@@ -1096,12 +1096,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Gold</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Platinum</t>
+          <t>Silver</t>
         </is>
       </c>
     </row>
@@ -1130,29 +1130,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HG</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Platinum</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CORECPI</t>
+          <t>HG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Copper</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CPI</t>
+          <t>CORECPI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CPI</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FEDFUNDS</t>
+          <t>CPI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Fed Funds Rate</t>
+          <t>CPI</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>FEDFUNDS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2-Year</t>
+          <t>Fed Funds Rate</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1215,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>US10Y</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10-Year</t>
+          <t>2-Year</t>
         </is>
       </c>
     </row>
@@ -1232,29 +1232,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>US30Y</t>
+          <t>US10Y</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>30-Year</t>
+          <t>10-Year</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TQQQ</t>
+          <t>US30Y</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>3x Nasdaq 100</t>
+          <t>30-Year</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1266,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>TQQQ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3x Semiconductors</t>
+          <t>3x Nasdaq 100</t>
         </is>
       </c>
     </row>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SPXL</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3x S&amp;P 500</t>
+          <t>3x Semiconductors</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>SPXL</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>3x Small-Cap</t>
+          <t>3x S&amp;P 500</t>
         </is>
       </c>
     </row>
@@ -1317,12 +1317,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>UDOW</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3x Dow Jones</t>
+          <t>3x Small-Cap</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TECL</t>
+          <t>UDOW</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>3x Technology</t>
+          <t>3x Dow Jones</t>
         </is>
       </c>
     </row>
@@ -1351,12 +1351,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>TECL</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2x Nasdaq 100</t>
+          <t>3x Technology</t>
         </is>
       </c>
     </row>
@@ -1368,12 +1368,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SSO</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2x S&amp;P 500</t>
+          <t>2x Nasdaq 100</t>
         </is>
       </c>
     </row>
@@ -1385,29 +1385,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>SSO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2x Semiconductors</t>
+          <t>2x S&amp;P 500</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>2x Semiconductors</t>
         </is>
       </c>
     </row>
@@ -1419,12 +1419,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Bitcoin</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Ethereum</t>
         </is>
       </c>
     </row>
@@ -1453,12 +1453,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>BNB</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Binance</t>
         </is>
       </c>
     </row>
@@ -1470,12 +1470,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Ripple</t>
         </is>
       </c>
     </row>
@@ -1487,12 +1487,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TRX</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Tron</t>
+          <t>Solana</t>
         </is>
       </c>
     </row>
@@ -1504,12 +1504,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>DOGE</t>
+          <t>TRX</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dogecoin</t>
+          <t>Tron</t>
         </is>
       </c>
     </row>
@@ -1521,12 +1521,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ZEC</t>
+          <t>DOGE</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Zcash</t>
+          <t>Dogecoin</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1538,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>ZEC</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Cardano</t>
+          <t>Zcash</t>
         </is>
       </c>
     </row>
@@ -1555,12 +1555,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>XMR</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Monero</t>
+          <t>Cardano</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>LTC</t>
+          <t>XMR</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Litecoin</t>
+          <t>Monero</t>
         </is>
       </c>
     </row>
@@ -1589,10 +1589,27 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>LTC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Litecoin</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>AVAX</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>

</xml_diff>